<commit_message>
Drop the naming point and remove statements about review status
- Remove the AI-native / agent naming point from findings, risks, controls,
  method documents, report and site (F-10 now covers the missing
  intended-use and limitations statement).
- Remove statements that the work had not been reviewed.
- Regenerate the remediation patch without the README wording change.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_risk/risk_register.xlsx
+++ b/02_risk/risk_register.xlsx
@@ -1538,7 +1538,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Reviewers over-rely on the tool because of the 'AI-native' label and the 7/7 headline</t>
+          <t>Reviewers over-rely on the tool because of the 7/7 headline</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>README.md:5; 7/7 claim</t>
+          <t>7/7 claim in the README and dashboard</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Ambiguous 'AI-native' and 'agent' positioning of a rules-based system: the README never says no model is used</t>
+          <t>Users are not told what the tool cannot detect, its known limits or that it is not for production use</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2313,12 +2313,12 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>README.md:5 positions the tool as a small-scale version of AI-native products; title says Agent; 'rule-based' only at line 108; no LLM (SysDesc s2); corrected in evidence log E-08</t>
+          <t>README has no intended-use or limitations statement; 'rule-based' only at line 108; no statement that no LLM is used (Phase 4, E-04)</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Present now. A reader can assume AI or adaptive behaviour; ambiguous positioning rather than a false claim.</t>
+          <t>Present now. Users could rely on the tool for more than it can do.</t>
         </is>
       </c>
     </row>

</xml_diff>